<commit_message>
Orgenized admin managing pages
</commit_message>
<xml_diff>
--- a/Data/Resources/example_users.xlsx
+++ b/Data/Resources/example_users.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26fc674a9d78ad98/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cyber_User\Programming\mentoringapp\Data\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_A422CFDA00232BA40AE6D2A899A3ED034E04A029" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96B4F634-37F8-40D5-A395-33F96B41BF69}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FF8A4CE-CC63-410D-8F28-D5BA63BBA1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3825" yWindow="3135" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -413,7 +413,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>111111111</v>
+        <v>666666666</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -424,7 +424,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>222222222</v>
+        <v>777777777</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>5</v>

</xml_diff>